<commit_message>
relatório formatados e novo botao de relatótio
</commit_message>
<xml_diff>
--- a/temp_op.xlsx
+++ b/temp_op.xlsx
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="R$#,##0.00"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -94,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -106,6 +108,10 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -473,18 +479,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="50.559" customWidth="1" min="2" max="2"/>
-    <col width="16.282" customWidth="1" min="3" max="3"/>
-    <col width="17.567" customWidth="1" min="4" max="4"/>
-    <col width="15.139" customWidth="1" min="5" max="5"/>
-    <col width="9.282999999999999" customWidth="1" min="6" max="6"/>
-    <col width="13.997" customWidth="1" min="7" max="7"/>
-    <col width="16.282" customWidth="1" min="8" max="8"/>
-    <col width="15.139" customWidth="1" min="9" max="9"/>
+    <col width="50.56" customWidth="1" min="2" max="2"/>
+    <col width="16.28" customWidth="1" min="3" max="3"/>
+    <col width="17.57" customWidth="1" min="4" max="4"/>
+    <col width="15.14" customWidth="1" min="5" max="5"/>
+    <col width="9.279999999999999" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16.28" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -500,12 +505,11 @@
       <c r="F1" s="2" t="n"/>
       <c r="G1" s="2" t="n"/>
       <c r="H1" s="2" t="n"/>
-      <c r="I1" s="2" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>SESP/DEPPEN – PAGAMENTO DE EXTRAJORNADA – REF. 06/2026 – REGIONAL DE UMUARAMA – PROTOCOLO 252</t>
+          <t>SESP/DEPPEN – PAGAMENTO DE EXTRAJORNADA – REF. 06/2026 – REGIONAL DE UMUARAMA – PROTOCOLO 2525</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -515,7 +519,6 @@
       <c r="F2" s="2" t="n"/>
       <c r="G2" s="2" t="n"/>
       <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -558,11 +561,6 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>Liquidação</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -572,118 +570,222 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>WILLIAN DOA SANTOS FORTES</t>
+          <t>PEDRO AUGUSTO DORNELAS DOS SANTOS</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>15942203792</t>
+          <t>05827685941</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026NE032824</t>
+          <t>2026NE032918</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>05/06/2026</t>
+          <t>15/06/2026</t>
         </is>
       </c>
       <c r="F4" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>R$ 180,00</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>R$ 360,00</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="n"/>
+      <c r="G4" s="5" t="n">
+        <v>180</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>180</v>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="n"/>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>PEG</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>REINALDO GONÇALVES PIRES</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>04732947964</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>2026NE032823</t>
+        </is>
+      </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>10/06/2026</t>
+          <t>09/06/2026</t>
         </is>
       </c>
       <c r="F5" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>360</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>PECO</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>RUBENS FARIAS</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>96633636522</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>2026NE032830</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>21/06/2026</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>R$ 180,00</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="n"/>
-      <c r="I5" s="5" t="n"/>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Total de Policiais: 1</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
-      <c r="H6" s="6" t="n"/>
-      <c r="I6" s="6" t="n"/>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Total de DEAEV: 2</t>
-        </is>
-      </c>
+      <c r="G6" s="5" t="n">
+        <v>180</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n"/>
       <c r="B7" s="6" t="n"/>
       <c r="C7" s="6" t="n"/>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="n"/>
-      <c r="H7" s="6" t="n"/>
-      <c r="I7" s="6" t="n"/>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>TOTAL de R$ 360,00</t>
-        </is>
-      </c>
+      <c r="D7" s="7" t="n"/>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>30/06/2026</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>360</v>
+      </c>
+      <c r="H7" s="7" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n"/>
       <c r="B8" s="6" t="n"/>
       <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="6" t="n"/>
-      <c r="H8" s="6" t="n"/>
-      <c r="I8" s="6" t="n"/>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>2026NE032836</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>03/06/2026</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>180</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="n"/>
+      <c r="B9" s="7" t="n"/>
+      <c r="C9" s="7" t="n"/>
+      <c r="D9" s="7" t="n"/>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>05/06/2026</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>360</v>
+      </c>
+      <c r="H9" s="7" t="n"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Total de Policiais: 3</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="n"/>
+      <c r="C10" s="8" t="n"/>
+      <c r="D10" s="8" t="n"/>
+      <c r="E10" s="8" t="n"/>
+      <c r="F10" s="8" t="n"/>
+      <c r="G10" s="8" t="n"/>
+      <c r="H10" s="8" t="n"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Total de DEAEV: 4,50</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="n"/>
+      <c r="C11" s="8" t="n"/>
+      <c r="D11" s="8" t="n"/>
+      <c r="E11" s="8" t="n"/>
+      <c r="F11" s="8" t="n"/>
+      <c r="G11" s="8" t="n"/>
+      <c r="H11" s="8" t="n"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL: R$ 1.620,00</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="n"/>
+      <c r="C12" s="8" t="n"/>
+      <c r="D12" s="8" t="n"/>
+      <c r="E12" s="8" t="n"/>
+      <c r="F12" s="8" t="n"/>
+      <c r="G12" s="8" t="n"/>
+      <c r="H12" s="8" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="A7:I7"/>
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="I4:I5"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A8:I8"/>
-    <mergeCell ref="A6:I6"/>
+  <mergeCells count="12">
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="H8:H9"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="H6:H7"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="B6:B9"/>
+    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="C6:C9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>